<commit_message>
Validated Income Tax utility JSON export for 3CA and 3CB
</commit_message>
<xml_diff>
--- a/clients/Ramya/AY 2026-27/Tax Audit Applicability/tax_audit_applicability_result.xlsx
+++ b/clients/Ramya/AY 2026-27/Tax Audit Applicability/tax_audit_applicability_result.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="63">
   <si>
     <t>Client Name</t>
   </si>
@@ -28,24 +28,36 @@
     <t>Activity Type</t>
   </si>
   <si>
+    <t>Business Nature</t>
+  </si>
+  <si>
+    <t>Is Resident</t>
+  </si>
+  <si>
+    <t>Detected Presumptive Section</t>
+  </si>
+  <si>
     <t>Presumptive Section</t>
   </si>
   <si>
-    <t>Presumptive Section Display</t>
-  </si>
-  <si>
-    <t>Business Nature</t>
-  </si>
-  <si>
-    <t>Is Resident</t>
+    <t>Presumptive Available</t>
+  </si>
+  <si>
+    <t>Presumptive Limit</t>
+  </si>
+  <si>
+    <t>Presumptive Limit Display</t>
+  </si>
+  <si>
+    <t>Exercise Presumptive Option</t>
+  </si>
+  <si>
+    <t>Earlier 44AD Opted / Lock-in Applicable</t>
   </si>
   <si>
     <t>Section 44AD(4) Applicable</t>
   </si>
   <si>
-    <t>Section 44AD(4) Display</t>
-  </si>
-  <si>
     <t>Turnover / Gross Receipts</t>
   </si>
   <si>
@@ -85,6 +97,12 @@
     <t>Declared Profit %</t>
   </si>
   <si>
+    <t>Presumptive Profit</t>
+  </si>
+  <si>
+    <t>Presumptive Profit Formatted</t>
+  </si>
+  <si>
     <t>44AD Presumptive Profit</t>
   </si>
   <si>
@@ -97,6 +115,9 @@
     <t>44ADA Presumptive Profit Formatted</t>
   </si>
   <si>
+    <t>Goods Carriages Owned</t>
+  </si>
+  <si>
     <t>Presumptive Profit 44AE</t>
   </si>
   <si>
@@ -127,6 +148,9 @@
     <t>Reason</t>
   </si>
   <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>Ramya</t>
   </si>
   <si>
@@ -139,58 +163,46 @@
     <t>Business</t>
   </si>
   <si>
+    <t>Eligible Business</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>44AD</t>
   </si>
   <si>
-    <t>44AD - Presumptive Taxation for Eligible Business</t>
-  </si>
-  <si>
-    <t>Eligible Business</t>
-  </si>
-  <si>
-    <t>Yes</t>
+    <t>₹3 crore</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>No - Section 44AD(4) not applicable</t>
-  </si>
-  <si>
-    <t>9,00,00,000</t>
-  </si>
-  <si>
-    <t>75,00,000</t>
-  </si>
-  <si>
-    <t>78,00,000</t>
-  </si>
-  <si>
-    <t>8,25,00,000</t>
-  </si>
-  <si>
-    <t>12,00,000</t>
-  </si>
-  <si>
-    <t>55,50,000</t>
-  </si>
-  <si>
-    <t>4,50,00,000</t>
-  </si>
-  <si>
-    <t>Presumptive Basis - Section 44AD</t>
+    <t>99,00,000</t>
+  </si>
+  <si>
+    <t>4,50,000</t>
+  </si>
+  <si>
+    <t>94,50,000</t>
+  </si>
+  <si>
+    <t>5,00,000</t>
+  </si>
+  <si>
+    <t>6,03,000</t>
+  </si>
+  <si>
+    <t>Normal Basis</t>
   </si>
   <si>
     <t>Not Applicable</t>
   </si>
   <si>
-    <t>ITR-4, subject to other ITR-4 eligibility conditions</t>
-  </si>
-  <si>
-    <t>Section 44AD</t>
-  </si>
-  <si>
-    <t>Accounts are not required to be audited under another law. If tax audit applies, Form 3CB-3CD will be applicable. | Presumptive profit under Section 44AD is ₹55,50,000 computed as 8% of cash turnover and 6% of digital/banking turnover. | Declared profit is lower than presumptive profit, but Section 44AB(e) condition is not triggered because either Section 44AD(4) is not applicable or income does not exceed basic exemption limit. | Since tax audit is not applicable, Form 3CA/3CB-3CD is not required.</t>
+    <t>ITR-3 for normal business/professional income</t>
+  </si>
+  <si>
+    <t>Accounts are not audited under another law. If tax audit applies, Form 3CB-3CD will be applicable. | Auto-detected presumptive section: 44AD. | Section 44AD is available because turnover is within ₹3 crore. | Presumptive taxation is available under Section 44AD, but the option is not exercised. | Business turnover is within applicable audit limit of ₹10,00,00,000. | Earlier 44AD lock-in condition is not selected. Special 44AD opt-out audit rule is not triggered. | Since tax audit is not applicable, Form 3CA/3CB-3CD is not required.</t>
   </si>
 </sst>
 </file>
@@ -522,10 +534,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:AS2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:37">
+    <row r="1" spans="1:45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -637,115 +649,157 @@
       <c r="AK1" t="s">
         <v>36</v>
       </c>
+      <c r="AL1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:37">
+    <row r="2" spans="1:45">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="H2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
-      </c>
-      <c r="J2" t="s">
-        <v>46</v>
-      </c>
-      <c r="K2">
-        <v>90000000</v>
+        <v>50</v>
+      </c>
+      <c r="J2">
+        <v>30000000</v>
+      </c>
+      <c r="K2" t="s">
+        <v>52</v>
       </c>
       <c r="L2" t="s">
-        <v>47</v>
-      </c>
-      <c r="M2">
-        <v>7500000</v>
+        <v>53</v>
+      </c>
+      <c r="M2" t="s">
+        <v>53</v>
       </c>
       <c r="N2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="O2">
-        <v>8.33</v>
-      </c>
-      <c r="P2">
-        <v>7800000</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>49</v>
-      </c>
-      <c r="R2">
-        <v>8.67</v>
+        <v>9900000</v>
+      </c>
+      <c r="P2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q2">
+        <v>450000</v>
+      </c>
+      <c r="R2" t="s">
+        <v>55</v>
       </c>
       <c r="S2">
-        <v>82500000</v>
-      </c>
-      <c r="T2" t="s">
+        <v>4.55</v>
+      </c>
+      <c r="T2">
+        <v>450000</v>
+      </c>
+      <c r="U2" t="s">
+        <v>55</v>
+      </c>
+      <c r="V2">
+        <v>4.55</v>
+      </c>
+      <c r="W2">
+        <v>9450000</v>
+      </c>
+      <c r="X2" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y2">
+        <v>500000</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA2">
+        <v>5.05</v>
+      </c>
+      <c r="AB2">
+        <v>603000</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD2">
+        <v>603000</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF2">
+        <v>0</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="s">
         <v>50</v>
       </c>
-      <c r="U2">
-        <v>1200000</v>
-      </c>
-      <c r="V2" t="s">
-        <v>51</v>
-      </c>
-      <c r="W2">
-        <v>1.33</v>
-      </c>
-      <c r="X2">
-        <v>5550000</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z2">
-        <v>45000000</v>
-      </c>
-      <c r="AA2" t="s">
+      <c r="AL2" t="s">
         <v>53</v>
       </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>54</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>55</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>57</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>58</v>
+      <c r="AM2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>